<commit_message>
change KIT ID from 9 to 19 (for RAK-GAN)
</commit_message>
<xml_diff>
--- a/Documents/Inbetriebnahme_DB42C02_14000_48V.xlsx
+++ b/Documents/Inbetriebnahme_DB42C02_14000_48V.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\RAK_GAN_RSS_GITHUB\RAK_GAN_MOTOR_DEMO\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83F8B930-506A-4524-9FF8-F0BDBDEB44A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FC2DF68-3A45-4002-98C3-643F92451C45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="76680" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{9AB2DC97-95DF-4ADE-8AE4-A797BFEF62A7}"/>
   </bookViews>
@@ -128,7 +128,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="701" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="702" uniqueCount="274">
   <si>
     <t>v_min</t>
   </si>
@@ -1425,6 +1425,9 @@
   </si>
   <si>
     <t>calc.</t>
+  </si>
+  <si>
+    <t>Ermittelt</t>
   </si>
 </sst>
 </file>
@@ -4547,7 +4550,9 @@
       <c r="P7" s="6"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="3"/>
-      <c r="S7" s="3"/>
+      <c r="S7" s="3" t="s">
+        <v>273</v>
+      </c>
     </row>
     <row r="8" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="3" t="s">

</xml_diff>